<commit_message>
Rebuild group 4 (Cabin extras) from the wire lists: CSB3, ClusterLED, AntiTheft, RearLights
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/CSB3-pinouts.xlsx
+++ b/docs/harness/wirelist/CSB3-pinouts.xlsx
@@ -1178,21 +1178,29 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>IN3</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr"/>
+          <t>IN2</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>w_sw7_c</t>
+        </is>
+      </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>spare, not used</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
+          <t>Reverse to opto in 2</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_rev_sw (SP-REV)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>IN4</t>
+          <t>IN3</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr"/>
@@ -1206,7 +1214,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>IN5</t>
+          <t>IN4</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr"/>
@@ -1220,7 +1228,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>IN6</t>
+          <t>IN5</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr"/>
@@ -1234,7 +1242,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>IN7</t>
+          <t>IN6</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr"/>
@@ -1248,7 +1256,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>IN8</t>
+          <t>IN7</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr"/>
@@ -1262,65 +1270,65 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>OUT1</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>w_opto_out1</t>
-        </is>
-      </c>
+          <t>IN8</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr"/>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Brake to CSB3 S7</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>CSB3 pin 21</t>
-        </is>
-      </c>
+          <t>spare, not used</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>OUT2</t>
+          <t>OUT1</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>w_opto_out2</t>
+          <t>w_opto_out1</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Reverse to CSB3 S8</t>
+          <t>Brake to CSB3 S7</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>CSB3 pin 22</t>
+          <t>CSB3 pin 21</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>OUT3</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr"/>
+          <t>OUT2</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>w_opto_out2</t>
+        </is>
+      </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>spare, not used</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr"/>
+          <t>Reverse to CSB3 S8</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>CSB3 pin 22</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>OUT4</t>
+          <t>OUT3</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr"/>
@@ -1334,7 +1342,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>OUT5</t>
+          <t>OUT4</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr"/>
@@ -1348,7 +1356,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>OUT6</t>
+          <t>OUT5</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr"/>
@@ -1362,7 +1370,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>OUT7</t>
+          <t>OUT6</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr"/>
@@ -1376,7 +1384,7 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>OUT8</t>
+          <t>OUT7</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr"/>
@@ -1390,44 +1398,36 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>VCC</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>w_opto_vcc</t>
-        </is>
-      </c>
+          <t>OUT8</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Opto +5 V</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>CSB3 pin 3</t>
-        </is>
-      </c>
+          <t>spare, not used</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>VCC</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>w_sw7_c</t>
+          <t>w_opto_vcc</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Reverse to opto in 2</t>
+          <t>Opto +5 V</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>splice sp_rev_sw (SP-REV)</t>
+          <t>CSB3 pin 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild group 4 (Cabin extras) from the wire lists: CSB3, ClusterLED, AntiTheft, RearLights (#345)
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/CSB3-pinouts.xlsx
+++ b/docs/harness/wirelist/CSB3-pinouts.xlsx
@@ -1178,21 +1178,29 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>IN3</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr"/>
+          <t>IN2</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>w_sw7_c</t>
+        </is>
+      </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>spare, not used</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
+          <t>Reverse to opto in 2</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_rev_sw (SP-REV)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>IN4</t>
+          <t>IN3</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr"/>
@@ -1206,7 +1214,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>IN5</t>
+          <t>IN4</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr"/>
@@ -1220,7 +1228,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>IN6</t>
+          <t>IN5</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr"/>
@@ -1234,7 +1242,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>IN7</t>
+          <t>IN6</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr"/>
@@ -1248,7 +1256,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>IN8</t>
+          <t>IN7</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr"/>
@@ -1262,65 +1270,65 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>OUT1</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>w_opto_out1</t>
-        </is>
-      </c>
+          <t>IN8</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr"/>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Brake to CSB3 S7</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>CSB3 pin 21</t>
-        </is>
-      </c>
+          <t>spare, not used</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>OUT2</t>
+          <t>OUT1</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>w_opto_out2</t>
+          <t>w_opto_out1</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Reverse to CSB3 S8</t>
+          <t>Brake to CSB3 S7</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>CSB3 pin 22</t>
+          <t>CSB3 pin 21</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>OUT3</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr"/>
+          <t>OUT2</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>w_opto_out2</t>
+        </is>
+      </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>spare, not used</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr"/>
+          <t>Reverse to CSB3 S8</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>CSB3 pin 22</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>OUT4</t>
+          <t>OUT3</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr"/>
@@ -1334,7 +1342,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>OUT5</t>
+          <t>OUT4</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr"/>
@@ -1348,7 +1356,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>OUT6</t>
+          <t>OUT5</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr"/>
@@ -1362,7 +1370,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>OUT7</t>
+          <t>OUT6</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr"/>
@@ -1376,7 +1384,7 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>OUT8</t>
+          <t>OUT7</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr"/>
@@ -1390,44 +1398,36 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>VCC</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>w_opto_vcc</t>
-        </is>
-      </c>
+          <t>OUT8</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Opto +5 V</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>CSB3 pin 3</t>
-        </is>
-      </c>
+          <t>spare, not used</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>VCC</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>w_sw7_c</t>
+          <t>w_opto_vcc</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Reverse to opto in 2</t>
+          <t>Opto +5 V</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>splice sp_rev_sw (SP-REV)</t>
+          <t>CSB3 pin 3</t>
         </is>
       </c>
     </row>

</xml_diff>